<commit_message>
Update live Hitter Tool data
</commit_message>
<xml_diff>
--- a/outputs/daily/hr_rankings_2026-06-21.xlsx
+++ b/outputs/daily/hr_rankings_2026-06-21.xlsx
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>64.5</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Elite Power, Strong Barrel, Premium Lineup Spot</t>
+          <t>Elite Power, Strong Barrel, Premium Lineup Spot, Hot Hitter/Streak</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -1657,7 +1657,7 @@
         <v>50</v>
       </c>
       <c r="U5" t="n">
-        <v>66.7</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -1709,22 +1709,22 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>Hot streak: 2 HR in last 7 games</t>
+          <t>Hot streak: 3 HR in last 7 games</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -3593,7 +3593,7 @@
         <v>80</v>
       </c>
       <c r="U12" t="n">
-        <v>57.8</v>
+        <v>56.2</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr">
@@ -4911,27 +4911,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>650489</t>
+          <t>680776</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-06-21T19:10:00Z</t>
+          <t>2026-06-21T20:10:00Z</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4941,17 +4941,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Jared Jones</t>
+          <t>Logan Gilbert</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>683003</t>
+          <t>669302</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -4974,26 +4974,26 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Premium Lineup Spot, Platoon Edge, Hot Hitter/Streak</t>
+          <t>Strong Barrel, Platoon Edge</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>27.2</v>
+        <v>41.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>52</v>
+        <v>54.9</v>
       </c>
       <c r="R17" t="n">
-        <v>66.7</v>
+        <v>56.4</v>
       </c>
       <c r="S17" t="n">
-        <v>100</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="T17" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="U17" t="n">
-        <v>72.7</v>
+        <v>23.4</v>
       </c>
       <c r="V17" t="inlineStr">
         <is>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -5028,7 +5028,7 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>H:2026/2025 P:2026</t>
+          <t>H:2026/2025 P:2026/2025</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr"/>
@@ -5045,27 +5045,27 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>Hot streak: 2 HR in last 7 games</t>
+          <t>Last 7 games: 4/26, 1 HR</t>
         </is>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>switch hitter; pitcher baseline 9.3% barrel, 4.0 HR allowed</t>
+          <t>platoon edge; pitcher baseline 10.8% barrel, 15.1 HR allowed</t>
         </is>
       </c>
       <c r="AM17" t="inlineStr">
@@ -5075,112 +5075,112 @@
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>5.87</t>
+          <t>11.03</t>
         </is>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>40.59</t>
+          <t>41.76</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>88.03</t>
+          <t>90.54</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
         <is>
-          <t>99.923</t>
+          <t>102.3517</t>
         </is>
       </c>
       <c r="AR17" t="inlineStr">
         <is>
-          <t>0.3617</t>
+          <t>0.3953</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>0.1295</t>
+          <t>0.1606</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>0.3025</t>
+          <t>0.3043</t>
         </is>
       </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>72.37</t>
+          <t>75.22</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>23.62</t>
+          <t>52.26</t>
         </is>
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>42.88</t>
+          <t>40.51</t>
         </is>
       </c>
       <c r="AX17" t="inlineStr">
         <is>
-          <t>30.9</t>
+          <t>21.39</t>
         </is>
       </c>
       <c r="AY17" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="AZ17" t="inlineStr">
         <is>
-          <t>0.1295</t>
+          <t>0.1783</t>
         </is>
       </c>
       <c r="BA17" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>10.84</t>
         </is>
       </c>
       <c r="BB17" t="inlineStr">
         <is>
-          <t>42.6</t>
+          <t>44.01</t>
         </is>
       </c>
       <c r="BC17" t="inlineStr">
         <is>
-          <t>89.7</t>
+          <t>90.73</t>
         </is>
       </c>
       <c r="BD17" t="inlineStr">
         <is>
-          <t>0.481</t>
+          <t>0.4041</t>
         </is>
       </c>
       <c r="BE17" t="inlineStr">
         <is>
-          <t>0.212</t>
+          <t>0.1729</t>
         </is>
       </c>
       <c r="BF17" t="inlineStr">
         <is>
-          <t>29.6</t>
+          <t>29.94</t>
         </is>
       </c>
       <c r="BG17" t="inlineStr">
         <is>
-          <t>In From LF</t>
+          <t>Out To RF</t>
         </is>
       </c>
       <c r="BH17" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>70</t>
         </is>
       </c>
       <c r="BI17" t="inlineStr">
         <is>
-          <t>Coors Field</t>
+          <t>T-Mobile Park</t>
         </is>
       </c>
       <c r="BJ17" t="inlineStr"/>
@@ -5191,47 +5191,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>680776</t>
+          <t>656811</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-06-21T20:10:00Z</t>
+          <t>2026-06-21T19:10:00Z</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Logan Gilbert</t>
+          <t>Michael Lorenzen</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>669302</t>
+          <t>547179</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>55.8</v>
+        <v>55.7</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -5254,26 +5254,26 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Strong Barrel, Platoon Edge</t>
+          <t>Premium Lineup Spot, Platoon Edge</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>41.4</v>
+        <v>33.7</v>
       </c>
       <c r="Q18" t="n">
-        <v>54.9</v>
+        <v>51.6</v>
       </c>
       <c r="R18" t="n">
-        <v>56.4</v>
+        <v>66.7</v>
       </c>
       <c r="S18" t="n">
-        <v>86.40000000000001</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="T18" t="n">
         <v>80</v>
       </c>
       <c r="U18" t="n">
-        <v>23.4</v>
+        <v>34.2</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -5325,12 +5325,12 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>31</t>
         </is>
       </c>
       <c r="AJ18" t="inlineStr">
@@ -5340,12 +5340,12 @@
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>Last 7 games: 4/26, 1 HR</t>
+          <t>Last 7 games: 7/31, 1 HR</t>
         </is>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>platoon edge; pitcher baseline 10.8% barrel, 15.1 HR allowed</t>
+          <t>platoon edge; pitcher baseline 9.0% barrel, 15.9 HR allowed</t>
         </is>
       </c>
       <c r="AM18" t="inlineStr">
@@ -5355,112 +5355,112 @@
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>11.03</t>
+          <t>6.69</t>
         </is>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>41.76</t>
+          <t>43.55</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>90.54</t>
+          <t>89.54</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>102.3517</t>
+          <t>99.5306</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>0.3953</t>
+          <t>0.4157</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>0.1606</t>
+          <t>0.1558</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>0.3043</t>
+          <t>0.3276</t>
         </is>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>75.22</t>
+          <t>71.03</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>52.26</t>
+          <t>12.06</t>
         </is>
       </c>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>40.51</t>
+          <t>36.42</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
         <is>
-          <t>21.39</t>
+          <t>28.08</t>
         </is>
       </c>
       <c r="AY18" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="AZ18" t="inlineStr">
         <is>
-          <t>0.1783</t>
+          <t>0.1728</t>
         </is>
       </c>
       <c r="BA18" t="inlineStr">
         <is>
-          <t>10.84</t>
+          <t>9.01</t>
         </is>
       </c>
       <c r="BB18" t="inlineStr">
         <is>
-          <t>44.01</t>
+          <t>43.61</t>
         </is>
       </c>
       <c r="BC18" t="inlineStr">
         <is>
-          <t>90.73</t>
+          <t>89.72</t>
         </is>
       </c>
       <c r="BD18" t="inlineStr">
         <is>
-          <t>0.4041</t>
+          <t>0.4699</t>
         </is>
       </c>
       <c r="BE18" t="inlineStr">
         <is>
-          <t>0.1729</t>
+          <t>0.1847</t>
         </is>
       </c>
       <c r="BF18" t="inlineStr">
         <is>
-          <t>29.94</t>
+          <t>25.59</t>
         </is>
       </c>
       <c r="BG18" t="inlineStr">
         <is>
-          <t>Out To RF</t>
+          <t>In From LF</t>
         </is>
       </c>
       <c r="BH18" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>88</t>
         </is>
       </c>
       <c r="BI18" t="inlineStr">
         <is>
-          <t>T-Mobile Park</t>
+          <t>Coors Field</t>
         </is>
       </c>
       <c r="BJ18" t="inlineStr"/>
@@ -5471,24 +5471,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>656811</t>
+          <t>650489</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>PIT</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>COL</t>
-        </is>
-      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>2026-06-21T19:10:00Z</t>
@@ -5496,22 +5496,22 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Michael Lorenzen</t>
+          <t>Jared Jones</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>547179</t>
+          <t>683003</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -5534,26 +5534,26 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Premium Lineup Spot, Platoon Edge</t>
+          <t>Premium Lineup Spot, Platoon Edge, Hot Hitter/Streak</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>33.7</v>
+        <v>27.2</v>
       </c>
       <c r="Q19" t="n">
-        <v>51.6</v>
+        <v>52</v>
       </c>
       <c r="R19" t="n">
         <v>66.7</v>
       </c>
       <c r="S19" t="n">
-        <v>94.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="T19" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="U19" t="n">
-        <v>34.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -5588,7 +5588,7 @@
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>H:2026/2025 P:2026/2025</t>
+          <t>H:2026/2025 P:2026</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr"/>
@@ -5605,27 +5605,27 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AI19" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>Last 7 games: 7/31, 1 HR</t>
+          <t>Hot streak: 2 HR in last 7 games</t>
         </is>
       </c>
       <c r="AL19" t="inlineStr">
         <is>
-          <t>platoon edge; pitcher baseline 9.0% barrel, 15.9 HR allowed</t>
+          <t>switch hitter; pitcher baseline 9.3% barrel, 4.0 HR allowed</t>
         </is>
       </c>
       <c r="AM19" t="inlineStr">
@@ -5635,97 +5635,97 @@
       </c>
       <c r="AN19" t="inlineStr">
         <is>
-          <t>6.69</t>
+          <t>5.87</t>
         </is>
       </c>
       <c r="AO19" t="inlineStr">
         <is>
-          <t>43.55</t>
+          <t>40.59</t>
         </is>
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>89.54</t>
+          <t>88.03</t>
         </is>
       </c>
       <c r="AQ19" t="inlineStr">
         <is>
-          <t>99.5306</t>
+          <t>99.923</t>
         </is>
       </c>
       <c r="AR19" t="inlineStr">
         <is>
-          <t>0.4157</t>
+          <t>0.3617</t>
         </is>
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>0.1558</t>
+          <t>0.1295</t>
         </is>
       </c>
       <c r="AT19" t="inlineStr">
         <is>
-          <t>0.3276</t>
+          <t>0.3025</t>
         </is>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>71.03</t>
+          <t>72.37</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>12.06</t>
+          <t>23.62</t>
         </is>
       </c>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>36.42</t>
+          <t>42.88</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr">
         <is>
-          <t>28.08</t>
+          <t>30.9</t>
         </is>
       </c>
       <c r="AY19" t="inlineStr">
         <is>
-          <t>12.8</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="AZ19" t="inlineStr">
         <is>
-          <t>0.1728</t>
+          <t>0.1295</t>
         </is>
       </c>
       <c r="BA19" t="inlineStr">
         <is>
-          <t>9.01</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="BB19" t="inlineStr">
         <is>
-          <t>43.61</t>
+          <t>42.6</t>
         </is>
       </c>
       <c r="BC19" t="inlineStr">
         <is>
-          <t>89.72</t>
+          <t>89.7</t>
         </is>
       </c>
       <c r="BD19" t="inlineStr">
         <is>
-          <t>0.4699</t>
+          <t>0.481</t>
         </is>
       </c>
       <c r="BE19" t="inlineStr">
         <is>
-          <t>0.1847</t>
+          <t>0.212</t>
         </is>
       </c>
       <c r="BF19" t="inlineStr">
         <is>
-          <t>25.59</t>
+          <t>29.6</t>
         </is>
       </c>
       <c r="BG19" t="inlineStr">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -9136,7 +9136,7 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>53.2</v>
+        <v>53.1</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -9169,7 +9169,7 @@
         <v>78</v>
       </c>
       <c r="U32" t="n">
-        <v>78.7</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="V32" t="inlineStr">
         <is>
@@ -9226,7 +9226,7 @@
       </c>
       <c r="AI32" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ32" t="inlineStr">
@@ -10203,22 +10203,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>605141</t>
+          <t>677594</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Julio Rodríguez</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -10233,22 +10233,22 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Brandon Young</t>
+          <t>Payton Tolle</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>687064</t>
+          <t>801139</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -10266,26 +10266,26 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Premium Lineup Spot, Hot Hitter/Streak</t>
+          <t>Premium Lineup Spot, Platoon Edge</t>
         </is>
       </c>
       <c r="P36" t="n">
-        <v>33.4</v>
+        <v>47.1</v>
       </c>
       <c r="Q36" t="n">
-        <v>42.1</v>
+        <v>24.8</v>
       </c>
       <c r="R36" t="n">
-        <v>61.6</v>
+        <v>56.4</v>
       </c>
       <c r="S36" t="n">
-        <v>94.90000000000001</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="T36" t="n">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="U36" t="n">
-        <v>72.7</v>
+        <v>25.3</v>
       </c>
       <c r="V36" t="inlineStr">
         <is>
@@ -10299,7 +10299,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -10337,142 +10337,142 @@
       </c>
       <c r="AH36" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AI36" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AJ36" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AK36" t="inlineStr">
         <is>
-          <t>Hot streak: 2 HR in last 7 games</t>
+          <t>Last 7 games: 4/24, 1 HR</t>
         </is>
       </c>
       <c r="AL36" t="inlineStr">
         <is>
-          <t>same-side matchup; pitcher baseline 8.0% barrel, 7.8 HR allowed</t>
+          <t>platoon edge; pitcher baseline 6.0% barrel, 5.0 HR allowed</t>
         </is>
       </c>
       <c r="AM36" t="inlineStr">
         <is>
-          <t>fly-ball profile; pitcher fly-ball pressure modest</t>
+          <t>neutral batted-ball profile; pitcher fly-ball pressure modest</t>
         </is>
       </c>
       <c r="AN36" t="inlineStr">
         <is>
-          <t>7.46</t>
+          <t>9.38</t>
         </is>
       </c>
       <c r="AO36" t="inlineStr">
         <is>
-          <t>36.5</t>
+          <t>44.85</t>
         </is>
       </c>
       <c r="AP36" t="inlineStr">
         <is>
-          <t>89.59</t>
+          <t>90.54</t>
         </is>
       </c>
       <c r="AQ36" t="inlineStr">
         <is>
-          <t>98.2946</t>
+          <t>102.8449</t>
         </is>
       </c>
       <c r="AR36" t="inlineStr">
         <is>
-          <t>0.4318</t>
+          <t>0.4685</t>
         </is>
       </c>
       <c r="AS36" t="inlineStr">
         <is>
-          <t>0.1595</t>
+          <t>0.2034</t>
         </is>
       </c>
       <c r="AT36" t="inlineStr">
         <is>
-          <t>0.3342</t>
+          <t>0.3419</t>
         </is>
       </c>
       <c r="AU36" t="inlineStr">
         <is>
-          <t>69.35</t>
+          <t>76.54</t>
         </is>
       </c>
       <c r="AV36" t="inlineStr">
         <is>
-          <t>8.07</t>
+          <t>66.28</t>
         </is>
       </c>
       <c r="AW36" t="inlineStr">
         <is>
-          <t>40.59</t>
+          <t>36.25</t>
         </is>
       </c>
       <c r="AX36" t="inlineStr">
         <is>
-          <t>36.6</t>
+          <t>25.28</t>
         </is>
       </c>
       <c r="AY36" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="AZ36" t="inlineStr">
         <is>
-          <t>0.1711</t>
+          <t>0.1916</t>
         </is>
       </c>
       <c r="BA36" t="inlineStr">
         <is>
-          <t>8.03</t>
+          <t>5.98</t>
         </is>
       </c>
       <c r="BB36" t="inlineStr">
         <is>
-          <t>41.57</t>
+          <t>34.52</t>
         </is>
       </c>
       <c r="BC36" t="inlineStr">
         <is>
-          <t>89.19</t>
+          <t>87.73</t>
         </is>
       </c>
       <c r="BD36" t="inlineStr">
         <is>
-          <t>0.4215</t>
+          <t>0.3469</t>
         </is>
       </c>
       <c r="BE36" t="inlineStr">
         <is>
-          <t>0.1707</t>
+          <t>0.131</t>
         </is>
       </c>
       <c r="BF36" t="inlineStr">
         <is>
-          <t>26.17</t>
+          <t>28.44</t>
         </is>
       </c>
       <c r="BG36" t="inlineStr">
         <is>
-          <t>Out To CF</t>
+          <t>Out To RF</t>
         </is>
       </c>
       <c r="BH36" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>70</t>
         </is>
       </c>
       <c r="BI36" t="inlineStr">
         <is>
-          <t>UNIQLO Field at Dodger Stadium</t>
+          <t>T-Mobile Park</t>
         </is>
       </c>
       <c r="BJ36" t="inlineStr"/>
@@ -10483,22 +10483,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>677594</t>
+          <t>681624</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Julio Rodríguez</t>
+          <t>Andy Pages</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BAL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -10513,26 +10513,26 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Payton Tolle</t>
+          <t>Brandon Young</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>801139</t>
+          <t>687064</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="L37" t="n">
-        <v>51.8</v>
+        <v>51.7</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -10546,26 +10546,26 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Premium Lineup Spot, Platoon Edge</t>
+          <t>Premium Lineup Spot</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>47.1</v>
+        <v>40.6</v>
       </c>
       <c r="Q37" t="n">
-        <v>24.8</v>
+        <v>42.1</v>
       </c>
       <c r="R37" t="n">
-        <v>56.4</v>
+        <v>61.6</v>
       </c>
       <c r="S37" t="n">
-        <v>96.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="T37" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="U37" t="n">
-        <v>25.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="V37" t="inlineStr">
         <is>
@@ -10579,7 +10579,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -10617,27 +10617,27 @@
       </c>
       <c r="AH37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AI37" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>28</t>
         </is>
       </c>
       <c r="AJ37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AK37" t="inlineStr">
         <is>
-          <t>Last 7 games: 4/24, 1 HR</t>
+          <t>Last 7 games: 5/28, 0 HR</t>
         </is>
       </c>
       <c r="AL37" t="inlineStr">
         <is>
-          <t>platoon edge; pitcher baseline 6.0% barrel, 5.0 HR allowed</t>
+          <t>same-side matchup; pitcher baseline 8.0% barrel, 7.8 HR allowed</t>
         </is>
       </c>
       <c r="AM37" t="inlineStr">
@@ -10647,112 +10647,112 @@
       </c>
       <c r="AN37" t="inlineStr">
         <is>
-          <t>9.38</t>
+          <t>8.75</t>
         </is>
       </c>
       <c r="AO37" t="inlineStr">
         <is>
-          <t>44.85</t>
+          <t>43.92</t>
         </is>
       </c>
       <c r="AP37" t="inlineStr">
         <is>
-          <t>90.54</t>
+          <t>89.23</t>
         </is>
       </c>
       <c r="AQ37" t="inlineStr">
         <is>
-          <t>102.8449</t>
+          <t>100.4685</t>
         </is>
       </c>
       <c r="AR37" t="inlineStr">
         <is>
-          <t>0.4685</t>
+          <t>0.4539</t>
         </is>
       </c>
       <c r="AS37" t="inlineStr">
         <is>
-          <t>0.2034</t>
+          <t>0.1819</t>
         </is>
       </c>
       <c r="AT37" t="inlineStr">
         <is>
-          <t>0.3419</t>
+          <t>0.3342</t>
         </is>
       </c>
       <c r="AU37" t="inlineStr">
         <is>
-          <t>76.54</t>
+          <t>72.81</t>
         </is>
       </c>
       <c r="AV37" t="inlineStr">
         <is>
-          <t>66.28</t>
+          <t>24.93</t>
         </is>
       </c>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>36.25</t>
+          <t>35.87</t>
         </is>
       </c>
       <c r="AX37" t="inlineStr">
         <is>
-          <t>25.28</t>
+          <t>28.37</t>
         </is>
       </c>
       <c r="AY37" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>18.6</t>
         </is>
       </c>
       <c r="AZ37" t="inlineStr">
         <is>
-          <t>0.1916</t>
+          <t>0.2086</t>
         </is>
       </c>
       <c r="BA37" t="inlineStr">
         <is>
-          <t>5.98</t>
+          <t>8.03</t>
         </is>
       </c>
       <c r="BB37" t="inlineStr">
         <is>
-          <t>34.52</t>
+          <t>41.57</t>
         </is>
       </c>
       <c r="BC37" t="inlineStr">
         <is>
-          <t>87.73</t>
+          <t>89.19</t>
         </is>
       </c>
       <c r="BD37" t="inlineStr">
         <is>
-          <t>0.3469</t>
+          <t>0.4215</t>
         </is>
       </c>
       <c r="BE37" t="inlineStr">
         <is>
-          <t>0.131</t>
+          <t>0.1707</t>
         </is>
       </c>
       <c r="BF37" t="inlineStr">
         <is>
-          <t>28.44</t>
+          <t>26.17</t>
         </is>
       </c>
       <c r="BG37" t="inlineStr">
         <is>
-          <t>Out To RF</t>
+          <t>Out To CF</t>
         </is>
       </c>
       <c r="BH37" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>74</t>
         </is>
       </c>
       <c r="BI37" t="inlineStr">
         <is>
-          <t>T-Mobile Park</t>
+          <t>UNIQLO Field at Dodger Stadium</t>
         </is>
       </c>
       <c r="BJ37" t="inlineStr"/>
@@ -10763,12 +10763,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>681624</t>
+          <t>605141</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Andy Pages</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -10793,7 +10793,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -10826,11 +10826,11 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Premium Lineup Spot</t>
+          <t>Premium Lineup Spot, Hot Hitter/Streak</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>40.6</v>
+        <v>33.4</v>
       </c>
       <c r="Q38" t="n">
         <v>42.1</v>
@@ -10839,13 +10839,13 @@
         <v>61.6</v>
       </c>
       <c r="S38" t="n">
-        <v>100</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="T38" t="n">
         <v>50</v>
       </c>
       <c r="U38" t="n">
-        <v>8.800000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="V38" t="inlineStr">
         <is>
@@ -10859,7 +10859,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -10897,22 +10897,22 @@
       </c>
       <c r="AH38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AI38" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AK38" t="inlineStr">
         <is>
-          <t>Last 7 games: 5/28, 0 HR</t>
+          <t>Hot streak: 2 HR in last 7 games</t>
         </is>
       </c>
       <c r="AL38" t="inlineStr">
@@ -10922,37 +10922,37 @@
       </c>
       <c r="AM38" t="inlineStr">
         <is>
-          <t>neutral batted-ball profile; pitcher fly-ball pressure modest</t>
+          <t>fly-ball profile; pitcher fly-ball pressure modest</t>
         </is>
       </c>
       <c r="AN38" t="inlineStr">
         <is>
-          <t>8.75</t>
+          <t>7.46</t>
         </is>
       </c>
       <c r="AO38" t="inlineStr">
         <is>
-          <t>43.92</t>
+          <t>36.5</t>
         </is>
       </c>
       <c r="AP38" t="inlineStr">
         <is>
-          <t>89.23</t>
+          <t>89.59</t>
         </is>
       </c>
       <c r="AQ38" t="inlineStr">
         <is>
-          <t>100.4685</t>
+          <t>98.2946</t>
         </is>
       </c>
       <c r="AR38" t="inlineStr">
         <is>
-          <t>0.4539</t>
+          <t>0.4318</t>
         </is>
       </c>
       <c r="AS38" t="inlineStr">
         <is>
-          <t>0.1819</t>
+          <t>0.1595</t>
         </is>
       </c>
       <c r="AT38" t="inlineStr">
@@ -10962,32 +10962,32 @@
       </c>
       <c r="AU38" t="inlineStr">
         <is>
-          <t>72.81</t>
+          <t>69.35</t>
         </is>
       </c>
       <c r="AV38" t="inlineStr">
         <is>
-          <t>24.93</t>
+          <t>8.07</t>
         </is>
       </c>
       <c r="AW38" t="inlineStr">
         <is>
-          <t>35.87</t>
+          <t>40.59</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr">
         <is>
-          <t>28.37</t>
+          <t>36.6</t>
         </is>
       </c>
       <c r="AY38" t="inlineStr">
         <is>
-          <t>18.6</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="AZ38" t="inlineStr">
         <is>
-          <t>0.2086</t>
+          <t>0.1711</t>
         </is>
       </c>
       <c r="BA38" t="inlineStr">
@@ -11628,7 +11628,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -12468,7 +12468,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -16060,7 +16060,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -19136,7 +19136,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -21096,7 +21096,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -21660,7 +21660,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -23028,7 +23028,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -26397,7 +26397,7 @@
         <v>78</v>
       </c>
       <c r="U94" t="n">
-        <v>40.7</v>
+        <v>39.2</v>
       </c>
       <c r="V94" t="inlineStr">
         <is>
@@ -26454,7 +26454,7 @@
       </c>
       <c r="AI94" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="AJ94" t="inlineStr">
@@ -26464,7 +26464,7 @@
       </c>
       <c r="AK94" t="inlineStr">
         <is>
-          <t>Last 7 games: 7/26, 1 HR</t>
+          <t>Last 7 games: 7/27, 1 HR</t>
         </is>
       </c>
       <c r="AL94" t="inlineStr">
@@ -26620,7 +26620,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -27964,7 +27964,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -31906,7 +31906,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>64.5</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -31920,7 +31920,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Elite Power, Strong Barrel, Premium Lineup Spot</t>
+          <t>Elite Power, Strong Barrel, Premium Lineup Spot, Hot Hitter/Streak</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -31939,7 +31939,7 @@
         <v>50</v>
       </c>
       <c r="U5" t="n">
-        <v>66.7</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -31991,22 +31991,22 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>Hot streak: 2 HR in last 7 games</t>
+          <t>Hot streak: 3 HR in last 7 games</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
@@ -32162,7 +32162,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -32442,7 +32442,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -33875,7 +33875,7 @@
         <v>80</v>
       </c>
       <c r="U12" t="n">
-        <v>57.8</v>
+        <v>56.2</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -33932,7 +33932,7 @@
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr">
@@ -35193,27 +35193,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>650489</t>
+          <t>680776</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Willi Castro</t>
+          <t>Jarren Duran</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-06-21T19:10:00Z</t>
+          <t>2026-06-21T20:10:00Z</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -35223,17 +35223,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Jared Jones</t>
+          <t>Logan Gilbert</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>683003</t>
+          <t>669302</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -35256,26 +35256,26 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Premium Lineup Spot, Platoon Edge, Hot Hitter/Streak</t>
+          <t>Strong Barrel, Platoon Edge</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>27.2</v>
+        <v>41.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>52</v>
+        <v>54.9</v>
       </c>
       <c r="R17" t="n">
-        <v>66.7</v>
+        <v>56.4</v>
       </c>
       <c r="S17" t="n">
-        <v>100</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="T17" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="U17" t="n">
-        <v>72.7</v>
+        <v>23.4</v>
       </c>
       <c r="V17" t="inlineStr">
         <is>
@@ -35289,7 +35289,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -35310,7 +35310,7 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>H:2026/2025 P:2026</t>
+          <t>H:2026/2025 P:2026/2025</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr"/>
@@ -35327,27 +35327,27 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>Hot streak: 2 HR in last 7 games</t>
+          <t>Last 7 games: 4/26, 1 HR</t>
         </is>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>switch hitter; pitcher baseline 9.3% barrel, 4.0 HR allowed</t>
+          <t>platoon edge; pitcher baseline 10.8% barrel, 15.1 HR allowed</t>
         </is>
       </c>
       <c r="AM17" t="inlineStr">
@@ -35357,112 +35357,112 @@
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>5.87</t>
+          <t>11.03</t>
         </is>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>40.59</t>
+          <t>41.76</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>88.03</t>
+          <t>90.54</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
         <is>
-          <t>99.923</t>
+          <t>102.3517</t>
         </is>
       </c>
       <c r="AR17" t="inlineStr">
         <is>
-          <t>0.3617</t>
+          <t>0.3953</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>0.1295</t>
+          <t>0.1606</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>0.3025</t>
+          <t>0.3043</t>
         </is>
       </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>72.37</t>
+          <t>75.22</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>23.62</t>
+          <t>52.26</t>
         </is>
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>42.88</t>
+          <t>40.51</t>
         </is>
       </c>
       <c r="AX17" t="inlineStr">
         <is>
-          <t>30.9</t>
+          <t>21.39</t>
         </is>
       </c>
       <c r="AY17" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="AZ17" t="inlineStr">
         <is>
-          <t>0.1295</t>
+          <t>0.1783</t>
         </is>
       </c>
       <c r="BA17" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>10.84</t>
         </is>
       </c>
       <c r="BB17" t="inlineStr">
         <is>
-          <t>42.6</t>
+          <t>44.01</t>
         </is>
       </c>
       <c r="BC17" t="inlineStr">
         <is>
-          <t>89.7</t>
+          <t>90.73</t>
         </is>
       </c>
       <c r="BD17" t="inlineStr">
         <is>
-          <t>0.481</t>
+          <t>0.4041</t>
         </is>
       </c>
       <c r="BE17" t="inlineStr">
         <is>
-          <t>0.212</t>
+          <t>0.1729</t>
         </is>
       </c>
       <c r="BF17" t="inlineStr">
         <is>
-          <t>29.6</t>
+          <t>29.94</t>
         </is>
       </c>
       <c r="BG17" t="inlineStr">
         <is>
-          <t>In From LF</t>
+          <t>Out To RF</t>
         </is>
       </c>
       <c r="BH17" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>70</t>
         </is>
       </c>
       <c r="BI17" t="inlineStr">
         <is>
-          <t>Coors Field</t>
+          <t>T-Mobile Park</t>
         </is>
       </c>
       <c r="BJ17" t="inlineStr"/>
@@ -35473,47 +35473,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>680776</t>
+          <t>656811</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jarren Duran</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-06-21T20:10:00Z</t>
+          <t>2026-06-21T19:10:00Z</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Logan Gilbert</t>
+          <t>Michael Lorenzen</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>669302</t>
+          <t>547179</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -35522,7 +35522,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>55.8</v>
+        <v>55.7</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -35536,26 +35536,26 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Strong Barrel, Platoon Edge</t>
+          <t>Premium Lineup Spot, Platoon Edge</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>41.4</v>
+        <v>33.7</v>
       </c>
       <c r="Q18" t="n">
-        <v>54.9</v>
+        <v>51.6</v>
       </c>
       <c r="R18" t="n">
-        <v>56.4</v>
+        <v>66.7</v>
       </c>
       <c r="S18" t="n">
-        <v>86.40000000000001</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="T18" t="n">
         <v>80</v>
       </c>
       <c r="U18" t="n">
-        <v>23.4</v>
+        <v>34.2</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
@@ -35569,7 +35569,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -35607,12 +35607,12 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>31</t>
         </is>
       </c>
       <c r="AJ18" t="inlineStr">
@@ -35622,12 +35622,12 @@
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>Last 7 games: 4/26, 1 HR</t>
+          <t>Last 7 games: 7/31, 1 HR</t>
         </is>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>platoon edge; pitcher baseline 10.8% barrel, 15.1 HR allowed</t>
+          <t>platoon edge; pitcher baseline 9.0% barrel, 15.9 HR allowed</t>
         </is>
       </c>
       <c r="AM18" t="inlineStr">
@@ -35637,112 +35637,112 @@
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>11.03</t>
+          <t>6.69</t>
         </is>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>41.76</t>
+          <t>43.55</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>90.54</t>
+          <t>89.54</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>102.3517</t>
+          <t>99.5306</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>0.3953</t>
+          <t>0.4157</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>0.1606</t>
+          <t>0.1558</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>0.3043</t>
+          <t>0.3276</t>
         </is>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>75.22</t>
+          <t>71.03</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>52.26</t>
+          <t>12.06</t>
         </is>
       </c>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>40.51</t>
+          <t>36.42</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
         <is>
-          <t>21.39</t>
+          <t>28.08</t>
         </is>
       </c>
       <c r="AY18" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="AZ18" t="inlineStr">
         <is>
-          <t>0.1783</t>
+          <t>0.1728</t>
         </is>
       </c>
       <c r="BA18" t="inlineStr">
         <is>
-          <t>10.84</t>
+          <t>9.01</t>
         </is>
       </c>
       <c r="BB18" t="inlineStr">
         <is>
-          <t>44.01</t>
+          <t>43.61</t>
         </is>
       </c>
       <c r="BC18" t="inlineStr">
         <is>
-          <t>90.73</t>
+          <t>89.72</t>
         </is>
       </c>
       <c r="BD18" t="inlineStr">
         <is>
-          <t>0.4041</t>
+          <t>0.4699</t>
         </is>
       </c>
       <c r="BE18" t="inlineStr">
         <is>
-          <t>0.1729</t>
+          <t>0.1847</t>
         </is>
       </c>
       <c r="BF18" t="inlineStr">
         <is>
-          <t>29.94</t>
+          <t>25.59</t>
         </is>
       </c>
       <c r="BG18" t="inlineStr">
         <is>
-          <t>Out To RF</t>
+          <t>In From LF</t>
         </is>
       </c>
       <c r="BH18" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>88</t>
         </is>
       </c>
       <c r="BI18" t="inlineStr">
         <is>
-          <t>T-Mobile Park</t>
+          <t>Coors Field</t>
         </is>
       </c>
       <c r="BJ18" t="inlineStr"/>
@@ -35753,24 +35753,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>656811</t>
+          <t>650489</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Willi Castro</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>PIT</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>COL</t>
-        </is>
-      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>2026-06-21T19:10:00Z</t>
@@ -35778,22 +35778,22 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Michael Lorenzen</t>
+          <t>Jared Jones</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>547179</t>
+          <t>683003</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -35816,26 +35816,26 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Premium Lineup Spot, Platoon Edge</t>
+          <t>Premium Lineup Spot, Platoon Edge, Hot Hitter/Streak</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>33.7</v>
+        <v>27.2</v>
       </c>
       <c r="Q19" t="n">
-        <v>51.6</v>
+        <v>52</v>
       </c>
       <c r="R19" t="n">
         <v>66.7</v>
       </c>
       <c r="S19" t="n">
-        <v>94.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="T19" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="U19" t="n">
-        <v>34.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
@@ -35849,7 +35849,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -35870,7 +35870,7 @@
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>H:2026/2025 P:2026/2025</t>
+          <t>H:2026/2025 P:2026</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr"/>
@@ -35887,27 +35887,27 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AI19" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>26</t>
         </is>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>Last 7 games: 7/31, 1 HR</t>
+          <t>Hot streak: 2 HR in last 7 games</t>
         </is>
       </c>
       <c r="AL19" t="inlineStr">
         <is>
-          <t>platoon edge; pitcher baseline 9.0% barrel, 15.9 HR allowed</t>
+          <t>switch hitter; pitcher baseline 9.3% barrel, 4.0 HR allowed</t>
         </is>
       </c>
       <c r="AM19" t="inlineStr">
@@ -35917,97 +35917,97 @@
       </c>
       <c r="AN19" t="inlineStr">
         <is>
-          <t>6.69</t>
+          <t>5.87</t>
         </is>
       </c>
       <c r="AO19" t="inlineStr">
         <is>
-          <t>43.55</t>
+          <t>40.59</t>
         </is>
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>89.54</t>
+          <t>88.03</t>
         </is>
       </c>
       <c r="AQ19" t="inlineStr">
         <is>
-          <t>99.5306</t>
+          <t>99.923</t>
         </is>
       </c>
       <c r="AR19" t="inlineStr">
         <is>
-          <t>0.4157</t>
+          <t>0.3617</t>
         </is>
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>0.1558</t>
+          <t>0.1295</t>
         </is>
       </c>
       <c r="AT19" t="inlineStr">
         <is>
-          <t>0.3276</t>
+          <t>0.3025</t>
         </is>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>71.03</t>
+          <t>72.37</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>12.06</t>
+          <t>23.62</t>
         </is>
       </c>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>36.42</t>
+          <t>42.88</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr">
         <is>
-          <t>28.08</t>
+          <t>30.9</t>
         </is>
       </c>
       <c r="AY19" t="inlineStr">
         <is>
-          <t>12.8</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="AZ19" t="inlineStr">
         <is>
-          <t>0.1728</t>
+          <t>0.1295</t>
         </is>
       </c>
       <c r="BA19" t="inlineStr">
         <is>
-          <t>9.01</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="BB19" t="inlineStr">
         <is>
-          <t>43.61</t>
+          <t>42.6</t>
         </is>
       </c>
       <c r="BC19" t="inlineStr">
         <is>
-          <t>89.72</t>
+          <t>89.7</t>
         </is>
       </c>
       <c r="BD19" t="inlineStr">
         <is>
-          <t>0.4699</t>
+          <t>0.481</t>
         </is>
       </c>
       <c r="BE19" t="inlineStr">
         <is>
-          <t>0.1847</t>
+          <t>0.212</t>
         </is>
       </c>
       <c r="BF19" t="inlineStr">
         <is>
-          <t>25.59</t>
+          <t>29.6</t>
         </is>
       </c>
       <c r="BG19" t="inlineStr">

</xml_diff>